<commit_message>
atz planilha com dados da OCOR X + 4 Atz com gráficos de grupos e atores ao longo do tempo
</commit_message>
<xml_diff>
--- a/relations_updated_20251103_000000.xlsx
+++ b/relations_updated_20251103_000000.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srest\PycharmProjects\Dashboard_Informacional2\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D5E40E-A8E5-4C02-A1FD-27A5E6C5E2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView minimized="1" xWindow="5460" yWindow="3360" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="relations_updated" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -142,11 +148,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -210,13 +216,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -254,7 +268,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -288,6 +302,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -322,9 +337,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -497,11 +513,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K33"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -536,7 +552,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>45964</v>
       </c>
@@ -565,7 +581,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45964</v>
       </c>
@@ -594,7 +610,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45964</v>
       </c>
@@ -623,7 +639,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45964</v>
       </c>
@@ -652,7 +668,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45964</v>
       </c>
@@ -681,7 +697,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45964</v>
       </c>
@@ -710,7 +726,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45964</v>
       </c>
@@ -739,7 +755,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45964</v>
       </c>
@@ -768,7 +784,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45964</v>
       </c>
@@ -797,7 +813,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>45964</v>
       </c>
@@ -826,7 +842,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>45964</v>
       </c>
@@ -855,7 +871,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>45964</v>
       </c>
@@ -884,7 +900,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>45964</v>
       </c>
@@ -913,7 +929,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>45964</v>
       </c>
@@ -942,7 +958,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>45964</v>
       </c>
@@ -971,7 +987,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>45964</v>
       </c>
@@ -1000,7 +1016,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>45964</v>
       </c>
@@ -1029,7 +1045,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>45964</v>
       </c>
@@ -1058,7 +1074,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>45964</v>
       </c>
@@ -1087,7 +1103,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>45964</v>
       </c>
@@ -1116,7 +1132,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45964</v>
       </c>
@@ -1145,7 +1161,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45964</v>
       </c>
@@ -1174,7 +1190,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45964</v>
       </c>
@@ -1203,7 +1219,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45964</v>
       </c>
@@ -1232,7 +1248,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45964</v>
       </c>
@@ -1261,7 +1277,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45964</v>
       </c>
@@ -1290,7 +1306,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45964</v>
       </c>
@@ -1319,7 +1335,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45964</v>
       </c>
@@ -1348,7 +1364,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45964</v>
       </c>
@@ -1377,7 +1393,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45964</v>
       </c>
@@ -1406,7 +1422,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45964</v>
       </c>
@@ -1435,7 +1451,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45964</v>
       </c>

</xml_diff>